<commit_message>
day1: project setup complete, libraries ready
Commit message: "day1: project setup complete, libraries ready"
Description:
- Project skeleton (folders, .gitignore, README)
- Altium project with 2 SchDoc, 1 PcbDoc, 2 Library
- PCB stackup 2L 1.6mm FR-4, basic DRC rules
- Libraries loaded: Pico H, TP4056, AO3401A, SS14, SRV05-4, JST-PH, 282834-2, SS12D00
- BOM_draft.xlsx with LCSC part numbers verified on JLCPCB
- Datasheets saved for all active components
</commit_message>
<xml_diff>
--- a/08-Pico-Limit-Switch-Shield/00_Docs/BOM_draft.xlsx
+++ b/08-Pico-Limit-Switch-Shield/00_Docs/BOM_draft.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\altium-learning-path\08-Pico-Limit-Switch-Shield\00_Docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53CFA02E-E019-47BE-ADB0-77BBCFF16E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -18,9 +24,317 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="101">
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>Value / Part</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Footprint</t>
+  </si>
+  <si>
+    <t>Manufacturer MPN</t>
+  </si>
+  <si>
+    <t>LCSC #</t>
+  </si>
+  <si>
+    <t>Basic/Ext</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>TP4056</t>
+  </si>
+  <si>
+    <t>AO3401A</t>
+  </si>
+  <si>
+    <t>SS14</t>
+  </si>
+  <si>
+    <t>S2B-PH-SM4-TB</t>
+  </si>
+  <si>
+    <t>Li-ion charger 1A</t>
+  </si>
+  <si>
+    <t>P-MOSFET, 4A, SOT-23</t>
+  </si>
+  <si>
+    <t>Schottky 1A 40V</t>
+  </si>
+  <si>
+    <t>Блок питания</t>
+  </si>
+  <si>
+    <t>JST-PH 2-pin SMD правый</t>
+  </si>
+  <si>
+    <t>SOP-8</t>
+  </si>
+  <si>
+    <t>SOT-23</t>
+  </si>
+  <si>
+    <t>SMA</t>
+  </si>
+  <si>
+    <t>JST_PH_2</t>
+  </si>
+  <si>
+    <t>S2B-PH-SM4-TB(LF)(SN)</t>
+  </si>
+  <si>
+    <t>Проверка LCSC-номеров: https://jlcpcb.com/parts</t>
+  </si>
+  <si>
+    <t>основа зарядки</t>
+  </si>
+  <si>
+    <t>power-path switch</t>
+  </si>
+  <si>
+    <t>USB → VSYS</t>
+  </si>
+  <si>
+    <t>разъём LiPo</t>
+  </si>
+  <si>
+    <t>Концевики и защита</t>
+  </si>
+  <si>
+    <t>J2–J6</t>
+  </si>
+  <si>
+    <t>D2–D6</t>
+  </si>
+  <si>
+    <t>Клеммник 2-pin винтовой</t>
+  </si>
+  <si>
+    <t>под концевики</t>
+  </si>
+  <si>
+    <t>защита GPIO</t>
+  </si>
+  <si>
+    <t>Индикация и управление</t>
+  </si>
+  <si>
+    <t>LED1</t>
+  </si>
+  <si>
+    <t>LED2</t>
+  </si>
+  <si>
+    <t>LED3</t>
+  </si>
+  <si>
+    <t>SW1</t>
+  </si>
+  <si>
+    <t>LED red 0603</t>
+  </si>
+  <si>
+    <t>LED green 0603</t>
+  </si>
+  <si>
+    <t>LED blue 0603</t>
+  </si>
+  <si>
+    <t>CHG (заряд)</t>
+  </si>
+  <si>
+    <t>STDBY (заряд завершён)</t>
+  </si>
+  <si>
+    <t>USER (пользовательский)</t>
+  </si>
+  <si>
+    <t>Slide switch SPDT</t>
+  </si>
+  <si>
+    <t>LED_0603</t>
+  </si>
+  <si>
+    <t>любой</t>
+  </si>
+  <si>
+    <t>от TP4056 pin CHRG</t>
+  </si>
+  <si>
+    <t>от TP4056 pin STDBY</t>
+  </si>
+  <si>
+    <t>GPIO Pico</t>
+  </si>
+  <si>
+    <t>вкл/выкл — опционально</t>
+  </si>
+  <si>
+    <t>MCU-модуль</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>P1, P2</t>
+  </si>
+  <si>
+    <t>Raspberry Pi Pico</t>
+  </si>
+  <si>
+    <t>Header 1×20 female</t>
+  </si>
+  <si>
+    <t>RP2040 module</t>
+  </si>
+  <si>
+    <t>2.54 mm 1 row</t>
+  </si>
+  <si>
+    <t>PICO_CASTELLATED</t>
+  </si>
+  <si>
+    <t>1×20_FEMALE</t>
+  </si>
+  <si>
+    <t>покупается отдельно</t>
+  </si>
+  <si>
+    <t>под Pico</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R3-R7</t>
+  </si>
+  <si>
+    <t>R8-R10</t>
+  </si>
+  <si>
+    <t>R11-R12</t>
+  </si>
+  <si>
+    <t>C1-C5</t>
+  </si>
+  <si>
+    <t>C6-C7</t>
+  </si>
+  <si>
+    <t>C8</t>
+  </si>
+  <si>
+    <t>Механика (не в BOM Altium, для себя)</t>
+  </si>
+  <si>
+    <t>винт M2.5×8 мм</t>
+  </si>
+  <si>
+    <t>стойка M2.5×11 мм</t>
+  </si>
+  <si>
+    <t>крепёж Pico к shield</t>
+  </si>
+  <si>
+    <t>1.2k (R_PROG для 1А) или 2k (500mA)</t>
+  </si>
+  <si>
+    <t>10k (gate pull-up/down)</t>
+  </si>
+  <si>
+    <t>10k (series для debounce)</t>
+  </si>
+  <si>
+    <t>1k (LED current limit)</t>
+  </si>
+  <si>
+    <t>1k (LED для TP4056)</t>
+  </si>
+  <si>
+    <t>100 nF (debounce + decoupling)</t>
+  </si>
+  <si>
+    <t>10 μF X5R (power rails)</t>
+  </si>
+  <si>
+    <t>4.7 μF X5R (TP4056 output)</t>
+  </si>
+  <si>
+    <t>0603</t>
+  </si>
+  <si>
+    <t>Пассивы (ориентировочные номиналы, уточним)</t>
+  </si>
+  <si>
+    <t>Альтернативы на часто меняющиеся позиции:</t>
+  </si>
+  <si>
+    <t>PESD3V3S1UB → ESD3V3U1U или SRV05-4 (4 канала в одном SOT-23-6, экономит место)</t>
+  </si>
+  <si>
+    <t>AO3401A → DMP2305U, SI2301, BSS84 (все P-MOSFET SOT-23)</t>
+  </si>
+  <si>
+    <t>SS14 → SS34, 1N5819 (все Schottky 1A, разные корпуса)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 282834-2</t>
+  </si>
+  <si>
+    <t>ESD TVS</t>
+  </si>
+  <si>
+    <t>SOT-23-6</t>
+  </si>
+  <si>
+    <t>SRV05-4.TCT</t>
+  </si>
+  <si>
+    <t>EG1218</t>
+  </si>
+  <si>
+    <t>SC0917</t>
+  </si>
+  <si>
+    <t>PBS-20</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +342,52 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -45,18 +395,132 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF00FFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -330,10 +794,732 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15" style="6" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="6"/>
+    <col min="3" max="3" width="26.5703125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="31.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="6"/>
+    <col min="8" max="8" width="11.7109375" style="6" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="6"/>
+    <col min="10" max="10" width="26.42578125" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="9"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="5">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="5"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="5"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="5">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="14"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="5">
+        <v>5</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="5">
+        <v>5</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="14"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="5">
+        <v>1</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="5"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="5">
+        <v>1</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="5"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="5">
+        <v>1</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="5"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="5">
+        <v>1</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="14"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="5">
+        <v>1</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="G16" s="5"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="5">
+        <v>2</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="G17" s="5"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="14"/>
+    </row>
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="5">
+        <v>1</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="5">
+        <v>1</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="5">
+        <v>5</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="5">
+        <v>3</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="5">
+        <v>2</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="5">
+        <v>5</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="5">
+        <v>2</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="5">
+        <v>1</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="14"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5">
+        <v>2</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5">
+        <v>2</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+      <c r="J33" s="11"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A35:J35"/>
+    <mergeCell ref="A36:J36"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A27:J27"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="E19:E26" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>